<commit_message>
feat: add new words
</commit_message>
<xml_diff>
--- a/data/Click Me (History Demo).xlsx
+++ b/data/Click Me (History Demo).xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Beginning of World War II</t>
   </si>
@@ -28,6 +28,9 @@
   </si>
   <si>
     <t>Einstein’s General Theory of Relativity</t>
+  </si>
+  <si>
+    <t>Opening of the Suez Canal</t>
   </si>
 </sst>
 </file>
@@ -63,8 +66,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -366,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -399,6 +403,14 @@
       </c>
       <c r="B4" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1869</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>